<commit_message>
Urlaubsplanung: echte Stationsliste (StäB, Station 1–7, sechs Tageskliniken)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01STi8KXZYJBp3Efpx2oTZR2
</commit_message>
<xml_diff>
--- a/urlaubsplanung/Urlaubswuensche_Kreativtherapie.xlsx
+++ b/urlaubsplanung/Urlaubswuensche_Kreativtherapie.xlsx
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="110">
   <si>
     <t xml:space="preserve">Urlaubswünsche Kreativtherapie – Jahresplanung</t>
   </si>
@@ -130,7 +130,7 @@
     <t xml:space="preserve">Einrichtung (einmalig, durch die verantwortliche Person)</t>
   </si>
   <si>
-    <t xml:space="preserve">1.  »Einstellungen«: Startdatum (B3), Fachrichtungen und Stationen mit Grenze »max. gleichzeitig weg«, Feiertage. Bundesweite Feiertage sind vorbelegt – Landesfeiertage und Schließtage ergänzen. Grenze leer = keine Grenze.</t>
+    <t xml:space="preserve">1.  »Einstellungen«: Startdatum (B3), Fachrichtungen und Stationen mit ihren Ampel-Werten (ab wie vielen Abwesenden gelb/hellrot/dunkelrot), Feiertage. Bundesweite Feiertage sind vorbelegt – Landesfeiertage und Schließtage ergänzen. Ampel-Werte leer: Station = Standardregel, Fachteam = keine Ampel.</t>
   </si>
   <si>
     <t xml:space="preserve">2.  »Team«: alle Therapeut:innen mit Fachrichtung, bis zu 4 Stationen und (optional) Urlaubsanspruch. Jeder Name nur einmal.</t>
@@ -241,7 +241,7 @@
     <t xml:space="preserve">Beispiel Finn</t>
   </si>
   <si>
-    <t xml:space="preserve">Station 1A wäre dann zu dünn – klären</t>
+    <t xml:space="preserve">Station 1 wäre dann zu dünn – klären</t>
   </si>
   <si>
     <t xml:space="preserve">Beispiel Gül</t>
@@ -286,16 +286,13 @@
     <t xml:space="preserve">Ergotherapie</t>
   </si>
   <si>
-    <t xml:space="preserve">Station 1A</t>
+    <t xml:space="preserve">StäB</t>
   </si>
   <si>
-    <t xml:space="preserve">Station 1B</t>
+    <t xml:space="preserve">TK Depression</t>
   </si>
   <si>
-    <t xml:space="preserve">Station 2A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tagesklinik</t>
+    <t xml:space="preserve">TK Sucht</t>
   </si>
   <si>
     <t xml:space="preserve">Musiktherapie</t>
@@ -377,16 +374,37 @@
     <t xml:space="preserve">Christi Himmelfahrt</t>
   </si>
   <si>
+    <t xml:space="preserve">Station 5</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pfingstmontag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Station 6</t>
   </si>
   <si>
     <t xml:space="preserve">Tag der Deutschen Einheit</t>
   </si>
   <si>
+    <t xml:space="preserve">Station 7</t>
+  </si>
+  <si>
     <t xml:space="preserve">1. Weihnachtstag</t>
   </si>
   <si>
+    <t xml:space="preserve">TK Migration</t>
+  </si>
+  <si>
     <t xml:space="preserve">2. Weihnachtstag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TK Psychosomatik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TK Allgemeinpsychiatrie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TK 55+</t>
   </si>
 </sst>
 </file>
@@ -16309,10 +16327,10 @@
         <v>70</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="E5" s="10"/>
       <c r="F5" s="10"/>
@@ -16341,9 +16359,11 @@
         <v>70</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="D6" s="10"/>
+        <v>63</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>71</v>
+      </c>
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
       <c r="G6" s="10" t="n">
@@ -16371,13 +16391,13 @@
         <v>70</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="F7" s="10"/>
       <c r="G7" s="10" t="n">
@@ -16402,13 +16422,13 @@
         <v>53</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
@@ -16434,13 +16454,13 @@
         <v>55</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C9" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D9" s="10" t="s">
         <v>72</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>63</v>
       </c>
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
@@ -16466,13 +16486,13 @@
         <v>56</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
@@ -16498,16 +16518,16 @@
         <v>58</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C11" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="E11" s="10" t="s">
         <v>72</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>63</v>
       </c>
       <c r="F11" s="10"/>
       <c r="G11" s="10" t="n">
@@ -17750,7 +17770,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -17769,7 +17789,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -17788,14 +17808,14 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="17" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B3" s="14" t="n">
         <v>46388</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -17811,7 +17831,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B4" s="18" t="n">
         <f aca="false">B3+365</f>
@@ -17834,7 +17854,7 @@
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1"/>
       <c r="B5" s="19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -17843,14 +17863,14 @@
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="19" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
       <c r="N5" s="20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O5" s="1"/>
     </row>
@@ -17859,42 +17879,42 @@
         <v>40</v>
       </c>
       <c r="B6" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="D6" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="E6" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="F6" s="9" t="s">
         <v>88</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>89</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="K6" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="L6" s="9" t="s">
         <v>90</v>
-      </c>
-      <c r="I6" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="J6" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="K6" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="L6" s="9" t="s">
-        <v>91</v>
       </c>
       <c r="M6" s="1"/>
       <c r="N6" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="O6" s="9" t="s">
         <v>92</v>
-      </c>
-      <c r="O6" s="9" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17922,19 +17942,19 @@
       <c r="K7" s="21"/>
       <c r="L7" s="22" t="n">
         <f aca="false">IF(H7="","",COUNTIF(Team!$C$5:$F$64,H7))</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M7" s="1"/>
       <c r="N7" s="14" t="n">
         <v>46388</v>
       </c>
       <c r="O7" s="15" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B8" s="21"/>
       <c r="C8" s="21"/>
@@ -17948,26 +17968,26 @@
       <c r="F8" s="24"/>
       <c r="G8" s="1"/>
       <c r="H8" s="15" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="I8" s="21"/>
       <c r="J8" s="21"/>
       <c r="K8" s="21"/>
       <c r="L8" s="22" t="n">
         <f aca="false">IF(H8="","",COUNTIF(Team!$C$5:$F$64,H8))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M8" s="1"/>
       <c r="N8" s="14" t="n">
         <v>46472</v>
       </c>
       <c r="O8" s="15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B9" s="21"/>
       <c r="C9" s="21"/>
@@ -17981,7 +18001,7 @@
       <c r="F9" s="25"/>
       <c r="G9" s="1"/>
       <c r="H9" s="15" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="I9" s="21"/>
       <c r="J9" s="21"/>
@@ -17995,12 +18015,12 @@
         <v>46475</v>
       </c>
       <c r="O9" s="15" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B10" s="21"/>
       <c r="C10" s="21"/>
@@ -18026,7 +18046,7 @@
         <v>46508</v>
       </c>
       <c r="O10" s="15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18041,21 +18061,21 @@
       <c r="F11" s="27"/>
       <c r="G11" s="1"/>
       <c r="H11" s="15" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="I11" s="21"/>
       <c r="J11" s="21"/>
       <c r="K11" s="21"/>
       <c r="L11" s="22" t="n">
         <f aca="false">IF(H11="","",COUNTIF(Team!$C$5:$F$64,H11))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M11" s="1"/>
       <c r="N11" s="14" t="n">
         <v>46513</v>
       </c>
       <c r="O11" s="15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18069,13 +18089,15 @@
       </c>
       <c r="F12" s="28"/>
       <c r="G12" s="1"/>
-      <c r="H12" s="15"/>
+      <c r="H12" s="15" t="s">
+        <v>99</v>
+      </c>
       <c r="I12" s="21"/>
       <c r="J12" s="21"/>
       <c r="K12" s="21"/>
-      <c r="L12" s="22" t="str">
+      <c r="L12" s="22" t="n">
         <f aca="false">IF(H12="","",COUNTIF(Team!$C$5:$F$64,H12))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M12" s="1"/>
       <c r="N12" s="14" t="n">
@@ -18096,20 +18118,22 @@
       </c>
       <c r="F13" s="29"/>
       <c r="G13" s="1"/>
-      <c r="H13" s="15"/>
+      <c r="H13" s="15" t="s">
+        <v>101</v>
+      </c>
       <c r="I13" s="21"/>
       <c r="J13" s="21"/>
       <c r="K13" s="21"/>
-      <c r="L13" s="22" t="str">
+      <c r="L13" s="22" t="n">
         <f aca="false">IF(H13="","",COUNTIF(Team!$C$5:$F$64,H13))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M13" s="1"/>
       <c r="N13" s="14" t="n">
         <v>46663</v>
       </c>
       <c r="O13" s="15" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18123,20 +18147,22 @@
       </c>
       <c r="F14" s="30"/>
       <c r="G14" s="1"/>
-      <c r="H14" s="15"/>
+      <c r="H14" s="15" t="s">
+        <v>103</v>
+      </c>
       <c r="I14" s="21"/>
       <c r="J14" s="21"/>
       <c r="K14" s="21"/>
-      <c r="L14" s="22" t="str">
+      <c r="L14" s="22" t="n">
         <f aca="false">IF(H14="","",COUNTIF(Team!$C$5:$F$64,H14))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M14" s="1"/>
       <c r="N14" s="14" t="n">
         <v>46746</v>
       </c>
       <c r="O14" s="15" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18150,20 +18176,22 @@
       </c>
       <c r="F15" s="31"/>
       <c r="G15" s="1"/>
-      <c r="H15" s="15"/>
+      <c r="H15" s="15" t="s">
+        <v>105</v>
+      </c>
       <c r="I15" s="21"/>
       <c r="J15" s="21"/>
       <c r="K15" s="21"/>
-      <c r="L15" s="22" t="str">
+      <c r="L15" s="22" t="n">
         <f aca="false">IF(H15="","",COUNTIF(Team!$C$5:$F$64,H15))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M15" s="1"/>
       <c r="N15" s="14" t="n">
         <v>46747</v>
       </c>
       <c r="O15" s="15" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18177,13 +18205,15 @@
       </c>
       <c r="F16" s="32"/>
       <c r="G16" s="1"/>
-      <c r="H16" s="15"/>
+      <c r="H16" s="15" t="s">
+        <v>73</v>
+      </c>
       <c r="I16" s="21"/>
       <c r="J16" s="21"/>
       <c r="K16" s="21"/>
-      <c r="L16" s="22" t="str">
+      <c r="L16" s="22" t="n">
         <f aca="false">IF(H16="","",COUNTIF(Team!$C$5:$F$64,H16))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="M16" s="1"/>
       <c r="N16" s="14"/>
@@ -18197,13 +18227,15 @@
       <c r="E17" s="33"/>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
-      <c r="H17" s="15"/>
+      <c r="H17" s="15" t="s">
+        <v>72</v>
+      </c>
       <c r="I17" s="21"/>
       <c r="J17" s="21"/>
       <c r="K17" s="21"/>
-      <c r="L17" s="22" t="str">
+      <c r="L17" s="22" t="n">
         <f aca="false">IF(H17="","",COUNTIF(Team!$C$5:$F$64,H17))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="M17" s="1"/>
       <c r="N17" s="14"/>
@@ -18217,13 +18249,15 @@
       <c r="E18" s="33"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
-      <c r="H18" s="15"/>
+      <c r="H18" s="15" t="s">
+        <v>107</v>
+      </c>
       <c r="I18" s="21"/>
       <c r="J18" s="21"/>
       <c r="K18" s="21"/>
-      <c r="L18" s="22" t="str">
+      <c r="L18" s="22" t="n">
         <f aca="false">IF(H18="","",COUNTIF(Team!$C$5:$F$64,H18))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M18" s="1"/>
       <c r="N18" s="14"/>
@@ -18237,13 +18271,15 @@
       <c r="E19" s="33"/>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
-      <c r="H19" s="15"/>
+      <c r="H19" s="15" t="s">
+        <v>108</v>
+      </c>
       <c r="I19" s="21"/>
       <c r="J19" s="21"/>
       <c r="K19" s="21"/>
-      <c r="L19" s="22" t="str">
+      <c r="L19" s="22" t="n">
         <f aca="false">IF(H19="","",COUNTIF(Team!$C$5:$F$64,H19))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M19" s="1"/>
       <c r="N19" s="14"/>
@@ -18257,13 +18293,15 @@
       <c r="E20" s="33"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
-      <c r="H20" s="15"/>
+      <c r="H20" s="15" t="s">
+        <v>109</v>
+      </c>
       <c r="I20" s="21"/>
       <c r="J20" s="21"/>
       <c r="K20" s="21"/>
-      <c r="L20" s="22" t="str">
+      <c r="L20" s="22" t="n">
         <f aca="false">IF(H20="","",COUNTIF(Team!$C$5:$F$64,H20))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M20" s="1"/>
       <c r="N20" s="14"/>

</xml_diff>

<commit_message>
Urlaubsplanung: Physiotherapie statt Kunsttherapie, Feiertage Baden-Württemberg
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01STi8KXZYJBp3Efpx2oTZR2
</commit_message>
<xml_diff>
--- a/urlaubsplanung/Urlaubswuensche_Kreativtherapie.xlsx
+++ b/urlaubsplanung/Urlaubswuensche_Kreativtherapie.xlsx
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="115">
   <si>
     <t xml:space="preserve">Urlaubswünsche Kreativtherapie – Jahresplanung</t>
   </si>
@@ -130,7 +130,7 @@
     <t xml:space="preserve">Einrichtung (einmalig, durch die verantwortliche Person)</t>
   </si>
   <si>
-    <t xml:space="preserve">1.  »Einstellungen«: Startdatum (B3), Fachrichtungen und Stationen mit ihren Ampel-Werten (ab wie vielen Abwesenden gelb/hellrot/dunkelrot), Feiertage. Bundesweite Feiertage sind vorbelegt – Landesfeiertage und Schließtage ergänzen. Ampel-Werte leer: Station = Standardregel, Fachteam = keine Ampel.</t>
+    <t xml:space="preserve">1.  »Einstellungen«: Startdatum (B3), Fachrichtungen und Stationen mit ihren Ampel-Werten (ab wie vielen Abwesenden gelb/hellrot/dunkelrot), Feiertage. Die Feiertage für Baden-Württemberg sind vorbelegt – Schließtage bei Bedarf ergänzen. Ampel-Werte leer: Station = Standardregel, Fachteam = keine Ampel.</t>
   </si>
   <si>
     <t xml:space="preserve">2.  »Team«: alle Therapeut:innen mit Fachrichtung, bis zu 4 Stationen und (optional) Urlaubsanspruch. Jeder Name nur einmal.</t>
@@ -247,6 +247,12 @@
     <t xml:space="preserve">Beispiel Gül</t>
   </si>
   <si>
+    <t xml:space="preserve">Beispiel Hana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pfingstferien</t>
+  </si>
+  <si>
     <t xml:space="preserve">Team</t>
   </si>
   <si>
@@ -301,6 +307,15 @@
     <t xml:space="preserve">Bewegungstherapie</t>
   </si>
   <si>
+    <t xml:space="preserve">Physiotherapie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Station 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TK 55+</t>
+  </si>
+  <si>
     <t xml:space="preserve">Einstellungen</t>
   </si>
   <si>
@@ -322,7 +337,7 @@
     <t xml:space="preserve">Station: leer = Standardregel</t>
   </si>
   <si>
-    <t xml:space="preserve">Bundesweite Feiertage vorbelegt – Landesfeiertage ergänzen!</t>
+    <t xml:space="preserve">Feiertage Baden-Württemberg vorbelegt – Schließtage ggf. ergänzen</t>
   </si>
   <si>
     <t xml:space="preserve">Gelb
@@ -359,13 +374,13 @@
     <t xml:space="preserve">Neujahr</t>
   </si>
   <si>
+    <t xml:space="preserve">Heilige Drei Könige</t>
+  </si>
+  <si>
     <t xml:space="preserve">Karfreitag</t>
   </si>
   <si>
     <t xml:space="preserve">Ostermontag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kunsttherapie</t>
   </si>
   <si>
     <t xml:space="preserve">Tag der Arbeit</t>
@@ -374,37 +389,37 @@
     <t xml:space="preserve">Christi Himmelfahrt</t>
   </si>
   <si>
-    <t xml:space="preserve">Station 5</t>
+    <t xml:space="preserve">Station 6</t>
   </si>
   <si>
     <t xml:space="preserve">Pfingstmontag</t>
   </si>
   <si>
-    <t xml:space="preserve">Station 6</t>
+    <t xml:space="preserve">Station 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fronleichnam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TK Migration</t>
   </si>
   <si>
     <t xml:space="preserve">Tag der Deutschen Einheit</t>
   </si>
   <si>
-    <t xml:space="preserve">Station 7</t>
+    <t xml:space="preserve">Allerheiligen</t>
   </si>
   <si>
     <t xml:space="preserve">1. Weihnachtstag</t>
   </si>
   <si>
-    <t xml:space="preserve">TK Migration</t>
+    <t xml:space="preserve">TK Psychosomatik</t>
   </si>
   <si>
     <t xml:space="preserve">2. Weihnachtstag</t>
   </si>
   <si>
-    <t xml:space="preserve">TK Psychosomatik</t>
-  </si>
-  <si>
     <t xml:space="preserve">TK Allgemeinpsychiatrie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TK 55+</t>
   </si>
 </sst>
 </file>
@@ -828,7 +843,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="26">
+  <dxfs count="27">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -881,6 +896,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF76B7B2"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9C755F"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -2011,26 +2034,36 @@
       <c r="J16" s="14"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="15"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
+      <c r="A17" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="11" t="n">
+        <v>46531</v>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>46542</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>60</v>
+      </c>
       <c r="F17" s="12" t="str">
         <f aca="false">IF($A17="","",IFERROR(INDEX(Team!$B$5:$B$64,MATCH($A17,Team!$A$5:$A$64,0)),"?"))</f>
-        <v/>
+        <v>Physiotherapie</v>
       </c>
       <c r="G17" s="13" t="str">
         <f aca="false">IF($A17="","",COUNTIF($A$6:$A17,$A17)&amp;". Wunsch")</f>
-        <v/>
-      </c>
-      <c r="H17" s="13" t="str">
+        <v>1. Wunsch</v>
+      </c>
+      <c r="H17" s="13" t="n">
         <f aca="false">IF(OR($A17="",$B17="",$C17="",$C17&lt;$B17),"",NETWORKDAYS($B17,$C17,Einstellungen!$N$7:$N$40))</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="I17" s="12" t="str">
         <f aca="false">IF($A17="","",IF(OR($B17="",$C17=""),"Von und Bis eintragen",IF($C17&lt;$B17,"Bis liegt vor Von",IF(ISNA(MATCH($A17,Team!$A$5:$A$64,0)),"Name fehlt im Blatt Team",IF(COUNTIFS($A$6:$A$605,$A17,$B$6:$B$605,"&lt;="&amp;$C17,$C$6:$C$605,"&gt;="&amp;$B17)&gt;1,"Überschneidet sich mit eigenem Wunsch",IF(OR($B17&lt;Einstellungen!$B$3,$C17&gt;Einstellungen!$B$4),"Teils außerhalb des Planungsjahres","ok"))))))</f>
-        <v/>
+        <v>ok</v>
       </c>
       <c r="J17" s="14"/>
     </row>
@@ -16149,47 +16182,47 @@
   </sheetData>
   <autoFilter ref="A5:J605"/>
   <conditionalFormatting sqref="A6:I605">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>$J6&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I6:I605">
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$I6="ok"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>AND($I6&lt;&gt;"",$I6&lt;&gt;"ok")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F6:F605">
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>AND($F6&lt;&gt;"",IFERROR(MATCH($F6,Einstellungen!$A$7:$A$16,0),0)=1)</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
       <formula>AND($F6&lt;&gt;"",IFERROR(MATCH($F6,Einstellungen!$A$7:$A$16,0),0)=2)</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>AND($F6&lt;&gt;"",IFERROR(MATCH($F6,Einstellungen!$A$7:$A$16,0),0)=3)</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>AND($F6&lt;&gt;"",IFERROR(MATCH($F6,Einstellungen!$A$7:$A$16,0),0)=4)</formula>
     </cfRule>
-    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
       <formula>AND($F6&lt;&gt;"",IFERROR(MATCH($F6,Einstellungen!$A$7:$A$16,0),0)=5)</formula>
     </cfRule>
-    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
+    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
       <formula>AND($F6&lt;&gt;"",IFERROR(MATCH($F6,Einstellungen!$A$7:$A$16,0),0)=6)</formula>
     </cfRule>
-    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
+    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="22">
       <formula>AND($F6&lt;&gt;"",IFERROR(MATCH($F6,Einstellungen!$A$7:$A$16,0),0)=7)</formula>
     </cfRule>
-    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="22">
+    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="23">
       <formula>AND($F6&lt;&gt;"",IFERROR(MATCH($F6,Einstellungen!$A$7:$A$16,0),0)=8)</formula>
     </cfRule>
-    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="23">
+    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="24">
       <formula>AND($F6&lt;&gt;"",IFERROR(MATCH($F6,Einstellungen!$A$7:$A$16,0),0)=9)</formula>
     </cfRule>
-    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="24">
+    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="25">
       <formula>AND($F6&lt;&gt;"",IFERROR(MATCH($F6,Einstellungen!$A$7:$A$16,0),0)=10)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16243,7 +16276,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -16258,7 +16291,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -16292,31 +16325,31 @@
         <v>40</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16324,13 +16357,13 @@
         <v>45</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E5" s="10"/>
       <c r="F5" s="10"/>
@@ -16356,13 +16389,13 @@
         <v>50</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
@@ -16388,16 +16421,16 @@
         <v>52</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F7" s="10"/>
       <c r="G7" s="10" t="n">
@@ -16422,13 +16455,13 @@
         <v>53</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
@@ -16454,13 +16487,13 @@
         <v>55</v>
       </c>
       <c r="B9" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="10" t="s">
         <v>74</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>72</v>
       </c>
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
@@ -16486,13 +16519,13 @@
         <v>56</v>
       </c>
       <c r="B10" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>75</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>73</v>
       </c>
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
@@ -16518,16 +16551,16 @@
         <v>58</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F11" s="10"/>
       <c r="G11" s="10" t="n">
@@ -16548,25 +16581,37 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="16" t="str">
+      <c r="A12" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="H12" s="10"/>
+      <c r="I12" s="16" t="n">
         <f aca="false">IF($A12="","",COUNTIF(Wünsche!$A$6:$A$605,$A12))</f>
-        <v/>
-      </c>
-      <c r="J12" s="16" t="str">
+        <v>1</v>
+      </c>
+      <c r="J12" s="16" t="n">
         <f aca="false">IF($A12="","",SUMIF(Wünsche!$A$6:$A$605,$A12,Wünsche!$H$6:$H$605))</f>
-        <v/>
-      </c>
-      <c r="K12" s="13" t="str">
+        <v>9</v>
+      </c>
+      <c r="K12" s="13" t="n">
         <f aca="false">IF(OR($A12="",G12=""),"",G12-J12)</f>
-        <v/>
+        <v>21</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17715,12 +17760,12 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="K5:K64">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="25">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="26">
       <formula>AND(K5&lt;&gt;"",K5&lt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:A64">
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="25">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="26">
       <formula>AND(A5&lt;&gt;"",COUNTIF($A$5:$A$64,A5)&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17770,7 +17815,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -17789,7 +17834,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -17808,14 +17853,14 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="17" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B3" s="14" t="n">
         <v>46388</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="8" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -17831,7 +17876,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B4" s="18" t="n">
         <f aca="false">B3+365</f>
@@ -17854,7 +17899,7 @@
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1"/>
       <c r="B5" s="19" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -17863,14 +17908,14 @@
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="19" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
       <c r="N5" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="O5" s="1"/>
     </row>
@@ -17879,47 +17924,47 @@
         <v>40</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="I6" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="I6" s="9" t="s">
-        <v>84</v>
-      </c>
       <c r="J6" s="9" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="L6" s="9" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="M6" s="1"/>
       <c r="N6" s="9" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="O6" s="9" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B7" s="21" t="n">
         <v>2</v>
@@ -17935,7 +17980,7 @@
       <c r="F7" s="23"/>
       <c r="G7" s="1"/>
       <c r="H7" s="15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I7" s="21"/>
       <c r="J7" s="21"/>
@@ -17949,12 +17994,12 @@
         <v>46388</v>
       </c>
       <c r="O7" s="15" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B8" s="21"/>
       <c r="C8" s="21"/>
@@ -17968,7 +18013,7 @@
       <c r="F8" s="24"/>
       <c r="G8" s="1"/>
       <c r="H8" s="15" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="I8" s="21"/>
       <c r="J8" s="21"/>
@@ -17979,15 +18024,15 @@
       </c>
       <c r="M8" s="1"/>
       <c r="N8" s="14" t="n">
-        <v>46472</v>
+        <v>46393</v>
       </c>
       <c r="O8" s="15" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B9" s="21"/>
       <c r="C9" s="21"/>
@@ -18001,7 +18046,7 @@
       <c r="F9" s="25"/>
       <c r="G9" s="1"/>
       <c r="H9" s="15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I9" s="21"/>
       <c r="J9" s="21"/>
@@ -18012,27 +18057,27 @@
       </c>
       <c r="M9" s="1"/>
       <c r="N9" s="14" t="n">
-        <v>46475</v>
+        <v>46472</v>
       </c>
       <c r="O9" s="15" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="B10" s="21"/>
       <c r="C10" s="21"/>
       <c r="D10" s="21"/>
       <c r="E10" s="22" t="n">
         <f aca="false">IF(A10="","",COUNTIF(Team!$B$5:$B$64,A10))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" s="26"/>
       <c r="G10" s="1"/>
       <c r="H10" s="15" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="I10" s="21"/>
       <c r="J10" s="21"/>
@@ -18043,10 +18088,10 @@
       </c>
       <c r="M10" s="1"/>
       <c r="N10" s="14" t="n">
-        <v>46508</v>
+        <v>46475</v>
       </c>
       <c r="O10" s="15" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18061,21 +18106,21 @@
       <c r="F11" s="27"/>
       <c r="G11" s="1"/>
       <c r="H11" s="15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I11" s="21"/>
       <c r="J11" s="21"/>
       <c r="K11" s="21"/>
       <c r="L11" s="22" t="n">
         <f aca="false">IF(H11="","",COUNTIF(Team!$C$5:$F$64,H11))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M11" s="1"/>
       <c r="N11" s="14" t="n">
-        <v>46513</v>
+        <v>46508</v>
       </c>
       <c r="O11" s="15" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18090,21 +18135,21 @@
       <c r="F12" s="28"/>
       <c r="G12" s="1"/>
       <c r="H12" s="15" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="I12" s="21"/>
       <c r="J12" s="21"/>
       <c r="K12" s="21"/>
       <c r="L12" s="22" t="n">
         <f aca="false">IF(H12="","",COUNTIF(Team!$C$5:$F$64,H12))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M12" s="1"/>
       <c r="N12" s="14" t="n">
-        <v>46524</v>
+        <v>46513</v>
       </c>
       <c r="O12" s="15" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18119,7 +18164,7 @@
       <c r="F13" s="29"/>
       <c r="G13" s="1"/>
       <c r="H13" s="15" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="I13" s="21"/>
       <c r="J13" s="21"/>
@@ -18130,10 +18175,10 @@
       </c>
       <c r="M13" s="1"/>
       <c r="N13" s="14" t="n">
-        <v>46663</v>
+        <v>46524</v>
       </c>
       <c r="O13" s="15" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18148,7 +18193,7 @@
       <c r="F14" s="30"/>
       <c r="G14" s="1"/>
       <c r="H14" s="15" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="I14" s="21"/>
       <c r="J14" s="21"/>
@@ -18159,10 +18204,10 @@
       </c>
       <c r="M14" s="1"/>
       <c r="N14" s="14" t="n">
-        <v>46746</v>
+        <v>46534</v>
       </c>
       <c r="O14" s="15" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18177,7 +18222,7 @@
       <c r="F15" s="31"/>
       <c r="G15" s="1"/>
       <c r="H15" s="15" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="I15" s="21"/>
       <c r="J15" s="21"/>
@@ -18188,10 +18233,10 @@
       </c>
       <c r="M15" s="1"/>
       <c r="N15" s="14" t="n">
-        <v>46747</v>
+        <v>46663</v>
       </c>
       <c r="O15" s="15" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18206,7 +18251,7 @@
       <c r="F16" s="32"/>
       <c r="G16" s="1"/>
       <c r="H16" s="15" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I16" s="21"/>
       <c r="J16" s="21"/>
@@ -18216,8 +18261,12 @@
         <v>2</v>
       </c>
       <c r="M16" s="1"/>
-      <c r="N16" s="14"/>
-      <c r="O16" s="15"/>
+      <c r="N16" s="14" t="n">
+        <v>46692</v>
+      </c>
+      <c r="O16" s="15" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1"/>
@@ -18228,7 +18277,7 @@
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="15" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I17" s="21"/>
       <c r="J17" s="21"/>
@@ -18238,8 +18287,12 @@
         <v>3</v>
       </c>
       <c r="M17" s="1"/>
-      <c r="N17" s="14"/>
-      <c r="O17" s="15"/>
+      <c r="N17" s="14" t="n">
+        <v>46746</v>
+      </c>
+      <c r="O17" s="15" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1"/>
@@ -18250,7 +18303,7 @@
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="15" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="I18" s="21"/>
       <c r="J18" s="21"/>
@@ -18260,8 +18313,12 @@
         <v>0</v>
       </c>
       <c r="M18" s="1"/>
-      <c r="N18" s="14"/>
-      <c r="O18" s="15"/>
+      <c r="N18" s="14" t="n">
+        <v>46747</v>
+      </c>
+      <c r="O18" s="15" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1"/>
@@ -18272,7 +18329,7 @@
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="15" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="I19" s="21"/>
       <c r="J19" s="21"/>
@@ -18294,14 +18351,14 @@
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="15" t="s">
-        <v>109</v>
+        <v>80</v>
       </c>
       <c r="I20" s="21"/>
       <c r="J20" s="21"/>
       <c r="K20" s="21"/>
       <c r="L20" s="22" t="n">
         <f aca="false">IF(H20="","",COUNTIF(Team!$C$5:$F$64,H20))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M20" s="1"/>
       <c r="N20" s="14"/>

</xml_diff>

<commit_message>
Urlaubsplanung: Theatertherapie ergänzt, Arbeitsdatei aus lokaler Namensliste erzeugbar
Echte Namen werden nur lokal verarbeitet (.gitignore), das Repository enthält weiter nur Beispieldaten.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01STi8KXZYJBp3Efpx2oTZR2
</commit_message>
<xml_diff>
--- a/urlaubsplanung/Urlaubswuensche_Kreativtherapie.xlsx
+++ b/urlaubsplanung/Urlaubswuensche_Kreativtherapie.xlsx
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="116">
   <si>
     <t xml:space="preserve">Urlaubswünsche Kreativtherapie – Jahresplanung</t>
   </si>
@@ -381,6 +381,9 @@
   </si>
   <si>
     <t xml:space="preserve">Ostermontag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Theatertherapie</t>
   </si>
   <si>
     <t xml:space="preserve">Tag der Arbeit</t>
@@ -18095,13 +18098,15 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15"/>
+      <c r="A11" s="15" t="s">
+        <v>102</v>
+      </c>
       <c r="B11" s="21"/>
       <c r="C11" s="21"/>
       <c r="D11" s="21"/>
-      <c r="E11" s="22" t="str">
+      <c r="E11" s="22" t="n">
         <f aca="false">IF(A11="","",COUNTIF(Team!$B$5:$B$64,A11))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F11" s="27"/>
       <c r="G11" s="1"/>
@@ -18120,7 +18125,7 @@
         <v>46508</v>
       </c>
       <c r="O11" s="15" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18149,7 +18154,7 @@
         <v>46513</v>
       </c>
       <c r="O12" s="15" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18164,7 +18169,7 @@
       <c r="F13" s="29"/>
       <c r="G13" s="1"/>
       <c r="H13" s="15" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I13" s="21"/>
       <c r="J13" s="21"/>
@@ -18178,7 +18183,7 @@
         <v>46524</v>
       </c>
       <c r="O13" s="15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18193,7 +18198,7 @@
       <c r="F14" s="30"/>
       <c r="G14" s="1"/>
       <c r="H14" s="15" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I14" s="21"/>
       <c r="J14" s="21"/>
@@ -18207,7 +18212,7 @@
         <v>46534</v>
       </c>
       <c r="O14" s="15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18222,7 +18227,7 @@
       <c r="F15" s="31"/>
       <c r="G15" s="1"/>
       <c r="H15" s="15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="I15" s="21"/>
       <c r="J15" s="21"/>
@@ -18236,7 +18241,7 @@
         <v>46663</v>
       </c>
       <c r="O15" s="15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18265,7 +18270,7 @@
         <v>46692</v>
       </c>
       <c r="O16" s="15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18291,7 +18296,7 @@
         <v>46746</v>
       </c>
       <c r="O17" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18303,7 +18308,7 @@
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I18" s="21"/>
       <c r="J18" s="21"/>
@@ -18317,7 +18322,7 @@
         <v>46747</v>
       </c>
       <c r="O18" s="15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18329,7 +18334,7 @@
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I19" s="21"/>
       <c r="J19" s="21"/>

</xml_diff>